<commit_message>
feat(locale_generator): test locale generation for new delta
</commit_message>
<xml_diff>
--- a/utils/localization/resources/backup/out_meta_5_20.xlsx
+++ b/utils/localization/resources/backup/out_meta_5_20.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nireshkumarr/Documents/ekstep/crowdsource-dataplatform/utils/localization/resources/backup/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sreejithv/TW/projects/ekStep/crowdsource-dataplatform/utils/localization/resources/backup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA7BA78-A2B0-9B44-A3B1-DA8EEC75AE13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A31E58D-B5B5-334B-BA7E-41351F989F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6446" uniqueCount="3799">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6578" uniqueCount="3801">
   <si>
     <t>Key</t>
   </si>
@@ -11458,6 +11458,52 @@
   </si>
   <si>
     <t>An unexpected error has occurred.</t>
+  </si>
+  <si>
+    <r>
+      <t>Translated &lt;contribution-count&gt; &lt;language&gt; &lt;span&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF4A86E8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>sentence(s)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>&lt;/span&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Validated &lt;validation-count&gt; &lt;language&gt; &lt;span&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF4A86E8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>sentence(s)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>&lt;/span&gt;</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -32059,6 +32105,39 @@
       <c r="B471" s="3" t="s">
         <v>3765</v>
       </c>
+      <c r="G471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="H471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="I471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="J471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="K471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="L471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="M471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="N471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="O471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="P471" s="3" t="s">
+        <v>3765</v>
+      </c>
+      <c r="Q471" s="3" t="s">
+        <v>3765</v>
+      </c>
     </row>
     <row r="472" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A472" s="2" t="s">
@@ -32067,6 +32146,39 @@
       <c r="B472" s="2" t="s">
         <v>3766</v>
       </c>
+      <c r="G472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="H472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="I472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="J472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="K472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="L472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="M472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="N472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="O472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="P472" s="2" t="s">
+        <v>3766</v>
+      </c>
+      <c r="Q472" s="2" t="s">
+        <v>3766</v>
+      </c>
     </row>
     <row r="473" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A473" s="2" t="s">
@@ -32075,6 +32187,39 @@
       <c r="B473" s="2" t="s">
         <v>3767</v>
       </c>
+      <c r="G473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="H473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="I473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="J473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="K473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="L473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="M473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="N473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="O473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="P473" s="2" t="s">
+        <v>3767</v>
+      </c>
+      <c r="Q473" s="2" t="s">
+        <v>3767</v>
+      </c>
     </row>
     <row r="474" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A474" s="2" t="s">
@@ -32083,6 +32228,39 @@
       <c r="B474" s="2" t="s">
         <v>3768</v>
       </c>
+      <c r="G474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="H474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="I474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="J474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="K474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="L474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="M474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="N474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="O474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="P474" s="2" t="s">
+        <v>3768</v>
+      </c>
+      <c r="Q474" s="2" t="s">
+        <v>3768</v>
+      </c>
     </row>
     <row r="475" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A475" s="3" t="s">
@@ -32091,6 +32269,39 @@
       <c r="B475" s="3" t="s">
         <v>3769</v>
       </c>
+      <c r="G475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="H475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="I475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="J475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="K475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="L475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="M475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="N475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="O475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="P475" s="3" t="s">
+        <v>3769</v>
+      </c>
+      <c r="Q475" s="3" t="s">
+        <v>3769</v>
+      </c>
     </row>
     <row r="476" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A476" s="3" t="s">
@@ -32099,20 +32310,119 @@
       <c r="B476" s="3" t="s">
         <v>3770</v>
       </c>
+      <c r="G476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="H476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="I476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="J476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="K476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="L476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="M476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="N476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="O476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="P476" s="3" t="s">
+        <v>3770</v>
+      </c>
+      <c r="Q476" s="3" t="s">
+        <v>3770</v>
+      </c>
     </row>
     <row r="477" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A477" s="3" t="s">
-        <v>3771</v>
+        <v>3799</v>
       </c>
       <c r="B477" s="3" t="s">
         <v>3771</v>
       </c>
+      <c r="G477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="H477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="I477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="J477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="K477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="L477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="M477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="N477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="O477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="P477" s="3" t="s">
+        <v>3771</v>
+      </c>
+      <c r="Q477" s="3" t="s">
+        <v>3771</v>
+      </c>
     </row>
     <row r="478" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A478" s="3" t="s">
+        <v>3800</v>
+      </c>
+      <c r="B478" s="3" t="s">
         <v>3772</v>
       </c>
-      <c r="B478" s="3" t="s">
+      <c r="G478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="H478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="I478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="J478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="K478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="L478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="M478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="N478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="O478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="P478" s="3" t="s">
+        <v>3772</v>
+      </c>
+      <c r="Q478" s="3" t="s">
         <v>3772</v>
       </c>
     </row>
@@ -32123,6 +32433,39 @@
       <c r="B479" s="3" t="s">
         <v>3796</v>
       </c>
+      <c r="G479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="H479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="I479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="J479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="K479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="L479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="M479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="N479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="O479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="P479" s="3" t="s">
+        <v>3796</v>
+      </c>
+      <c r="Q479" s="3" t="s">
+        <v>3796</v>
+      </c>
     </row>
     <row r="480" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A480" s="4" t="s">
@@ -32131,20 +32474,119 @@
       <c r="B480" s="4" t="s">
         <v>3797</v>
       </c>
-    </row>
-    <row r="481" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="G480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="H480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="I480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="J480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="K480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="L480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="M480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="N480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="O480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="P480" s="4" t="s">
+        <v>3797</v>
+      </c>
+      <c r="Q480" s="4" t="s">
+        <v>3797</v>
+      </c>
+    </row>
+    <row r="481" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A481" s="4" t="s">
         <v>3798</v>
       </c>
       <c r="B481" s="4" t="s">
         <v>3798</v>
       </c>
-    </row>
-    <row r="482" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="G481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="H481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="I481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="J481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="K481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="L481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="M481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="N481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="O481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="P481" s="4" t="s">
+        <v>3798</v>
+      </c>
+      <c r="Q481" s="4" t="s">
+        <v>3798</v>
+      </c>
+    </row>
+    <row r="482" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A482" s="4" t="s">
         <v>2871</v>
       </c>
       <c r="B482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="G482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="H482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="I482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="J482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="K482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="L482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="M482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="N482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="O482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="P482" s="4" t="s">
+        <v>2871</v>
+      </c>
+      <c r="Q482" s="4" t="s">
         <v>2871</v>
       </c>
     </row>

</xml_diff>